<commit_message>
DCH sheet update from run 36051171734
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -509,6 +509,132 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/customers</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>customers</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Customer Master</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>customer-data-team@example.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>One record per customer with home state, signup date, and plan tier.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>/Volumes/workspace/dch_demo/landing/customers/</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>546</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:35Z</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:52:58Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>36051171734</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/orders</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>orders</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Customer Orders</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>order-analytics-team@example.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>One record per order with customer ID, order date, and total in USD.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>/Volumes/workspace/dch_demo/landing/orders/</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>289</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:35Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:22Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>36051171734</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -520,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,6 +689,102 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:35Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/customers</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>{"data_product_name": {"old": null, "new": "Customer Master"}, "owner": {"old": null, "new": "customer-data-team@example.com"}, "domain": {"old": null, "new": "Sales"}, "description": {"old": null, "new": "One record per customer with home state, signup date, and plan tier."}, "file_count": {"old": null, "new": 2}, "total_bytes": {"old": null, "new": 546}, "last_updated": {"old": null, "new": "2026-09-24T19:52:58Z"}}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>36051171734</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>23f13518b75650ef25581c50c979de3d2e4eb86a</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:35Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/inventory</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>validation_failed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"missing": ["owner", "domain"]}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>36051171734</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>23f13518b75650ef25581c50c979de3d2e4eb86a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:53:35Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/orders</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{"data_product_name": {"old": null, "new": "Customer Orders"}, "owner": {"old": null, "new": "order-analytics-team@example.com"}, "domain": {"old": null, "new": "Commerce"}, "description": {"old": null, "new": "One record per order with customer ID, order date, and total in USD."}, "file_count": {"old": null, "new": 1}, "total_bytes": {"old": null, "new": 289}, "last_updated": {"old": null, "new": "2026-09-24T19:53:22Z"}}</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>36051171734</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>23f13518b75650ef25581c50c979de3d2e4eb86a</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DCH sheet update from run 36085574396
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>546</v>
+        <v>873</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -563,12 +563,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-24T19:52:58Z</t>
+          <t>2026-09-25T02:15:39Z</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>36051171734</t>
+          <t>36085574396</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -785,6 +785,38 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:16:34Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/customers</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{"file_count": {"old": 2, "new": 3}, "total_bytes": {"old": 546, "new": 873}, "last_updated": {"old": "2026-09-24T19:52:58Z", "new": "2026-09-25T02:15:39Z"}}</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>36085574396</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>c068c0873e683dbf59380a8efcd1cc9983e37aba</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DCH sheet update from run 36152719514
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>873</v>
+        <v>1092</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -563,12 +563,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-25T02:15:39Z</t>
+          <t>2026-09-25T15:13:08Z</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>36085574396</t>
+          <t>36152719514</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -817,6 +817,38 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:13:47Z</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/customers</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{"file_count": {"old": 3, "new": 4}, "total_bytes": {"old": 873, "new": 1092}, "last_updated": {"old": "2026-09-25T02:15:39Z", "new": "2026-09-25T15:13:08Z"}}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>36152719514</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>78a6a4df343eab881aea94501835512c83283761</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DCH sheet update from run 36153372585
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2" t="n">
-        <v>1092</v>
+        <v>1311</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -563,12 +563,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-25T15:13:08Z</t>
+          <t>2026-09-25T15:18:28Z</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>36152719514</t>
+          <t>36153372585</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -849,6 +849,38 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:19:35Z</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/customers</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{"file_count": {"old": 4, "new": 5}, "total_bytes": {"old": 1092, "new": 1311}, "last_updated": {"old": "2026-09-25T15:13:08Z", "new": "2026-09-25T15:18:28Z"}}</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>36153372585</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>e7090a86c0313f4fcef61030ae230fc0bd20696a</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DCH sheet update from run 36154048614
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -614,10 +614,10 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>289</v>
+        <v>578</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -626,12 +626,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-24T19:53:22Z</t>
+          <t>2026-09-25T15:24:59Z</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>36051171734</t>
+          <t>36154048614</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -881,6 +881,38 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:25:37Z</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/orders</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{"file_count": {"old": 1, "new": 2}, "total_bytes": {"old": 289, "new": 578}, "last_updated": {"old": "2026-09-24T19:53:22Z", "new": "2026-09-25T15:24:59Z"}}</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>36154048614</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>17bf5433196620518f6eb9532d3a283bee8b8975</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DCH sheet update from run 36157188516
</commit_message>
<xml_diff>
--- a/dch/dch_registry.xlsx
+++ b/dch/dch_registry.xlsx
@@ -614,10 +614,10 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>578</v>
+        <v>867</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -626,12 +626,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-25T15:24:59Z</t>
+          <t>2026-09-25T15:53:09Z</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>36154048614</t>
+          <t>36157188516</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,38 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-25T15:53:34Z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>urn:dch:dataset:databricks:dev:workspace.dch_demo.landing/orders</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{"file_count": {"old": 2, "new": 3}, "total_bytes": {"old": 578, "new": 867}, "last_updated": {"old": "2026-09-25T15:24:59Z", "new": "2026-09-25T15:53:09Z"}}</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>36157188516</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8956e0fdf4645b1a9e8ab0334d01b9e7d1268ab8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>